<commit_message>
Inclusão de atividades da aula 21092026
</commit_message>
<xml_diff>
--- a/AULA 21092026/ATIVIDADE EXCEL PTIC.xlsx
+++ b/AULA 21092026/ATIVIDADE EXCEL PTIC.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CAMARGO\Desktop\projetos_de_tecnologia_de_informacao_e_comunicacao\AULA 21092026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{94DBC0E9-C7B6-48FC-8266-5BF91320A68C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{596D5EF5-0D27-47C5-B844-D252CA65A982}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" xr2:uid="{1DAE4682-B86A-404A-A057-CC81811930FF}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="29">
   <si>
     <t>Aluno</t>
   </si>
@@ -97,6 +97,21 @@
   </si>
   <si>
     <t>soma</t>
+  </si>
+  <si>
+    <t>Nota3</t>
+  </si>
+  <si>
+    <t>Nota4</t>
+  </si>
+  <si>
+    <t>Nota Máximo</t>
+  </si>
+  <si>
+    <t>A nota máxima</t>
+  </si>
+  <si>
+    <t>Média</t>
   </si>
 </sst>
 </file>
@@ -167,9 +182,6 @@
   </cellStyleXfs>
   <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -177,6 +189,9 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -495,7 +510,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4796349C-7566-4668-8BFD-F82B257C12C5}">
-  <dimension ref="B2:X19"/>
+  <dimension ref="B2:Z19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="15.42578125" bestFit="1" customWidth="1"/>
@@ -503,10 +518,11 @@
     <col min="5" max="5" width="12.28515625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="10.7109375" customWidth="1"/>
     <col min="9" max="9" width="9.140625" customWidth="1"/>
+    <col min="10" max="10" width="14.28515625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B2" s="6" t="s">
         <v>18</v>
       </c>
@@ -516,55 +532,67 @@
       <c r="F2" s="6"/>
       <c r="G2" s="6"/>
     </row>
-    <row r="3" spans="2:24" x14ac:dyDescent="0.25">
-      <c r="B3" s="1" t="s">
+    <row r="3" spans="2:26" x14ac:dyDescent="0.25">
+      <c r="B3" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
-      <c r="J3" s="1" t="s">
+      <c r="C3" s="5"/>
+      <c r="D3" s="5"/>
+      <c r="E3" s="5"/>
+      <c r="F3" s="5"/>
+      <c r="G3" s="5"/>
+      <c r="J3" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="K3" s="1"/>
-      <c r="L3" s="1"/>
-      <c r="M3" s="1"/>
-    </row>
-    <row r="4" spans="2:24" x14ac:dyDescent="0.25">
-      <c r="B4" s="5" t="s">
+      <c r="K3" s="5"/>
+      <c r="L3" s="5"/>
+      <c r="M3" s="5"/>
+      <c r="N3" s="5"/>
+      <c r="O3" s="5"/>
+      <c r="P3" s="5"/>
+    </row>
+    <row r="4" spans="2:26" x14ac:dyDescent="0.25">
+      <c r="B4" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="F4" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="G4" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="J4" s="2" t="s">
+      <c r="J4" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="K4" s="2" t="s">
+      <c r="K4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="L4" s="2" t="s">
+      <c r="L4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="M4" s="2" t="s">
+      <c r="M4" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="N4" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O4" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="5" spans="2:24" x14ac:dyDescent="0.25">
+      <c r="P4" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="5" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>19</v>
       </c>
@@ -574,21 +602,31 @@
       <c r="D5" t="s">
         <v>15</v>
       </c>
-      <c r="J5" s="3" t="s">
+      <c r="J5" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="K5" s="3">
+      <c r="K5" s="2">
         <v>2</v>
       </c>
-      <c r="L5" s="3">
+      <c r="L5" s="2">
         <v>7</v>
       </c>
-      <c r="M5" s="3">
-        <f>K5+L5</f>
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" spans="2:24" x14ac:dyDescent="0.25">
+      <c r="M5" s="2">
+        <v>1</v>
+      </c>
+      <c r="N5" s="2">
+        <v>6</v>
+      </c>
+      <c r="O5" s="2">
+        <f>SUM(K5:N5)</f>
+        <v>16</v>
+      </c>
+      <c r="P5" s="2">
+        <f>AVERAGE(K5:N5)</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>20</v>
       </c>
@@ -598,21 +636,31 @@
       <c r="D6" t="s">
         <v>15</v>
       </c>
-      <c r="J6" s="3" t="s">
+      <c r="J6" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="K6" s="3">
+      <c r="K6" s="2">
         <v>8</v>
       </c>
-      <c r="L6" s="3">
+      <c r="L6" s="2">
         <v>5</v>
       </c>
-      <c r="M6" s="3">
-        <f t="shared" ref="M6:M9" si="0">K6+L6</f>
-        <v>13</v>
-      </c>
-    </row>
-    <row r="7" spans="2:24" x14ac:dyDescent="0.25">
+      <c r="M6" s="2">
+        <v>9</v>
+      </c>
+      <c r="N6" s="2">
+        <v>8</v>
+      </c>
+      <c r="O6" s="2">
+        <f t="shared" ref="O6:O9" si="0">SUM(K6:N6)</f>
+        <v>30</v>
+      </c>
+      <c r="P6" s="2">
+        <f t="shared" ref="P6:P9" si="1">AVERAGE(K6:N6)</f>
+        <v>7.5</v>
+      </c>
+    </row>
+    <row r="7" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>21</v>
       </c>
@@ -622,21 +670,31 @@
       <c r="D7" t="s">
         <v>15</v>
       </c>
-      <c r="J7" s="3" t="s">
+      <c r="J7" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="K7" s="3">
+      <c r="K7" s="2">
         <v>9</v>
       </c>
-      <c r="L7" s="3">
+      <c r="L7" s="2">
         <v>8</v>
       </c>
-      <c r="M7" s="3">
+      <c r="M7" s="2">
+        <v>2</v>
+      </c>
+      <c r="N7" s="2">
+        <v>7</v>
+      </c>
+      <c r="O7" s="2">
         <f t="shared" si="0"/>
-        <v>17</v>
-      </c>
-    </row>
-    <row r="8" spans="2:24" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+      <c r="P7" s="2">
+        <f t="shared" si="1"/>
+        <v>6.5</v>
+      </c>
+    </row>
+    <row r="8" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>23</v>
       </c>
@@ -646,58 +704,94 @@
       <c r="D8" t="s">
         <v>15</v>
       </c>
-      <c r="J8" s="3" t="s">
+      <c r="J8" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="K8" s="3">
+      <c r="K8" s="2">
         <v>10</v>
       </c>
-      <c r="L8" s="3">
+      <c r="L8" s="2">
         <v>3</v>
       </c>
-      <c r="M8" s="3">
+      <c r="M8" s="2">
+        <v>10</v>
+      </c>
+      <c r="N8" s="2">
+        <v>8</v>
+      </c>
+      <c r="O8" s="2">
         <f t="shared" si="0"/>
-        <v>13</v>
-      </c>
-    </row>
-    <row r="9" spans="2:24" x14ac:dyDescent="0.25">
-      <c r="J9" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="P8" s="2">
+        <f t="shared" si="1"/>
+        <v>7.75</v>
+      </c>
+    </row>
+    <row r="9" spans="2:26" x14ac:dyDescent="0.25">
+      <c r="J9" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="K9" s="3">
+      <c r="K9" s="2">
         <v>1</v>
       </c>
-      <c r="L9" s="3">
+      <c r="L9" s="2">
         <v>6</v>
       </c>
-      <c r="M9" s="3">
+      <c r="M9" s="2">
+        <v>5</v>
+      </c>
+      <c r="N9" s="2">
+        <v>3</v>
+      </c>
+      <c r="O9" s="2">
         <f t="shared" si="0"/>
-        <v>7</v>
-      </c>
-    </row>
-    <row r="14" spans="2:24" x14ac:dyDescent="0.25">
-      <c r="X14" s="4"/>
-    </row>
-    <row r="15" spans="2:24" x14ac:dyDescent="0.25">
-      <c r="X15" s="4"/>
-    </row>
-    <row r="16" spans="2:24" x14ac:dyDescent="0.25">
-      <c r="X16" s="4"/>
-    </row>
-    <row r="17" spans="24:24" x14ac:dyDescent="0.25">
-      <c r="X17" s="4"/>
-    </row>
-    <row r="18" spans="24:24" x14ac:dyDescent="0.25">
-      <c r="X18" s="4"/>
-    </row>
-    <row r="19" spans="24:24" x14ac:dyDescent="0.25">
-      <c r="X19" s="4"/>
+        <v>15</v>
+      </c>
+      <c r="P9" s="2">
+        <f t="shared" si="1"/>
+        <v>3.75</v>
+      </c>
+    </row>
+    <row r="13" spans="2:26" x14ac:dyDescent="0.25">
+      <c r="J13" t="s">
+        <v>27</v>
+      </c>
+      <c r="K13">
+        <f>MAX(K5:N9)</f>
+        <v>10</v>
+      </c>
+      <c r="M13" t="s">
+        <v>26</v>
+      </c>
+      <c r="O13">
+        <f>MAX(O5:O9)</f>
+        <v>31</v>
+      </c>
+    </row>
+    <row r="14" spans="2:26" x14ac:dyDescent="0.25">
+      <c r="Z14" s="3"/>
+    </row>
+    <row r="15" spans="2:26" x14ac:dyDescent="0.25">
+      <c r="Z15" s="3"/>
+    </row>
+    <row r="16" spans="2:26" x14ac:dyDescent="0.25">
+      <c r="Z16" s="3"/>
+    </row>
+    <row r="17" spans="26:26" x14ac:dyDescent="0.25">
+      <c r="Z17" s="3"/>
+    </row>
+    <row r="18" spans="26:26" x14ac:dyDescent="0.25">
+      <c r="Z18" s="3"/>
+    </row>
+    <row r="19" spans="26:26" x14ac:dyDescent="0.25">
+      <c r="Z19" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="J3:M3"/>
     <mergeCell ref="B2:G2"/>
     <mergeCell ref="B3:G3"/>
+    <mergeCell ref="J3:P3"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>